<commit_message>
Me voy a dormir
</commit_message>
<xml_diff>
--- a/data/generated/plots/GANsEvaluation.xlsx
+++ b/data/generated/plots/GANsEvaluation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,22 +537,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>96.86799999999999</v>
+        <v>99.387</v>
       </c>
       <c r="D4" t="n">
-        <v>6.432</v>
+        <v>6.486</v>
       </c>
       <c r="E4" t="n">
-        <v>0.272</v>
+        <v>0.347</v>
       </c>
       <c r="F4" t="n">
-        <v>83.53400000000001</v>
+        <v>82.639</v>
       </c>
       <c r="G4" t="n">
-        <v>5.951</v>
+        <v>5.896</v>
       </c>
       <c r="H4" t="n">
-        <v>0.467</v>
+        <v>0.495</v>
       </c>
     </row>
     <row r="5">
@@ -565,22 +565,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>172.534</v>
-      </c>
-      <c r="D5" t="n">
-        <v>6.458</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.505</v>
+        <v>173.811</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>6.637</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.631</v>
       </c>
       <c r="F5" t="n">
-        <v>134.439</v>
-      </c>
-      <c r="G5" t="n">
-        <v>5.956</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0.66</v>
+        <v>128.199</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>6.289</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.485</v>
       </c>
     </row>
     <row r="6">
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>201.747</v>
+        <v>200.036</v>
       </c>
       <c r="D6" t="n">
-        <v>6.034</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>1.034</v>
+        <v>6.278</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.289</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>197.535</v>
+        <v>196.421</v>
       </c>
       <c r="G6" t="n">
-        <v>5.685</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.549</v>
+        <v>5.897</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.525</v>
       </c>
     </row>
     <row r="7">
@@ -621,22 +621,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>97.258</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>6.722</v>
+        <v>99.642</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.564</v>
       </c>
       <c r="E7" t="n">
-        <v>0.428</v>
+        <v>0.374</v>
       </c>
       <c r="F7" t="n">
-        <v>83.902</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>6.138</v>
+        <v>85.107</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.195</v>
       </c>
       <c r="H7" t="n">
-        <v>0.116</v>
+        <v>0.306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>